<commit_message>
rover_platform_mbse: carry the variable rename into the SWRS sets and exports
The ROVER_<SCOPE>_<THING> rename (e5fb89d) updated the JSON seeds and hand-edited the SysML
export, but not the SWRS .slreqx sets, which are the masters from V-001 on, nor the xlsx
exports. Regenerating the exports therefore brought the old names back.

SWR-BRG-007/008/013, SWR-DESC-011, SWR-DIAG-009/013 and SWR-LOC-009/011/014 now take their
text from the seeds (only the variable names differ). Their Summaries are recomputed the way
build_requirements does. The regenerated SysML export differs from the committed one only in
the two Summaries the hand edit had left longer than the 90-character cut. It passes the
Pilot kernel. The xlsx exports with content changes are included (SWRS for BRG, DESC, DIAG,
LOC and the SYS-SR compliance workbook), with the DESC workbook also picking up
SWR-DESC-006/010 from the previous commit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rover_platform_mbse/export/ROVER-A1-ROVER_BRINGUP-SWRS-V-001.xlsx
+++ b/rover_platform_mbse/export/ROVER-A1-ROVER_BRINGUP-SWRS-V-001.xlsx
@@ -946,7 +946,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>The rover_bringup shall start rover_localization with use_ekf True and fuse_gps set from the use_gps argument (default $ROVER_USE_GPS, else false).</t>
+          <t>The rover_bringup shall start rover_localization with use_ekf True and fuse_gps set from the use_gps argument (default $ROVER_SYSTEM_USE_GPS, else false).</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>The rover_bringup shall pass namespace (default $ROVER_NAMESPACE, else empty), log_level (DEBUG/INFO/WARN/ERROR/FATAL, default INFO) and common_dir_path (default empty) to every included launch file.</t>
+          <t>The rover_bringup shall pass namespace (default $ROVER_SYSTEM_NAMESPACE, else empty), log_level (DEBUG/INFO/WARN/ERROR/FATAL, default INFO) and common_dir_path (default empty) to every included launch file.</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>The rover_bringup shall restrict foxglove_bridge to the whitelisted topics (/tf, /tf_static and the listed UI topics under any namespace) and to the whitelisted services, unless ROVER_FOXGLOVE_TOPIC_WHITELIST or ROVER_FOXGLOVE_SERVICE_WHITELIST is set non-empty.</t>
+          <t>The rover_bringup shall restrict foxglove_bridge to the whitelisted topics (/tf, /tf_static and the listed UI topics under any namespace) and to the whitelisted services, unless ROVER_PLATFORM_FOXGLOVE_TOPIC_WHITELIST or ROVER_PLATFORM_FOXGLOVE_SERVICE_WHITELIST is set non-empty.</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -1690,7 +1690,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">

</xml_diff>